<commit_message>
fix: enable Gmail SMTP by default on Vercel & local and expand auto-pilot window to 08:00-16:00 WITA
</commit_message>
<xml_diff>
--- a/data/pelanggan_agung_toyota_gianyar.xlsx
+++ b/data/pelanggan_agung_toyota_gianyar.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:Q2"/>
   <cols>
     <col min="1" max="1" width="5.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
@@ -409,12 +409,13 @@
     <col min="8" max="8" width="16.83203125" customWidth="1"/>
     <col min="9" max="9" width="18.83203125" customWidth="1"/>
     <col min="10" max="10" width="18.83203125" customWidth="1"/>
-    <col min="11" max="11" width="16.83203125" customWidth="1"/>
-    <col min="12" max="12" width="28.83203125" customWidth="1"/>
-    <col min="13" max="13" width="18.83203125" customWidth="1"/>
-    <col min="14" max="14" width="16.83203125" customWidth="1"/>
-    <col min="15" max="15" width="28.83203125" customWidth="1"/>
-    <col min="16" max="16" width="34.83203125" customWidth="1"/>
+    <col min="11" max="11" width="18.83203125" customWidth="1"/>
+    <col min="12" max="12" width="16.83203125" customWidth="1"/>
+    <col min="13" max="13" width="28.83203125" customWidth="1"/>
+    <col min="14" max="14" width="18.83203125" customWidth="1"/>
+    <col min="15" max="15" width="16.83203125" customWidth="1"/>
+    <col min="16" max="16" width="28.83203125" customWidth="1"/>
+    <col min="17" max="17" width="34.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -446,24 +447,27 @@
         <v>Tgl Expired Asuransi</v>
       </c>
       <c r="J1" t="str">
+        <v>Tgl Next Service</v>
+      </c>
+      <c r="K1" t="str">
         <v>Nama Sales</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>No. WA Sales</v>
       </c>
-      <c r="L1" t="str">
+      <c r="M1" t="str">
         <v>Email Sales</v>
       </c>
-      <c r="M1" t="str">
+      <c r="N1" t="str">
         <v>Nama SA</v>
       </c>
-      <c r="N1" t="str">
+      <c r="O1" t="str">
         <v>No. WA SA</v>
       </c>
-      <c r="O1" t="str">
+      <c r="P1" t="str">
         <v>Email SA</v>
       </c>
-      <c r="P1" t="str">
+      <c r="Q1" t="str">
         <v>Status Log Pengiriman</v>
       </c>
     </row>
@@ -496,30 +500,33 @@
         <v>2026-10-24</v>
       </c>
       <c r="J2" t="str">
+        <v>2026-10-27</v>
+      </c>
+      <c r="K2" t="str">
         <v>I Made Putra</v>
       </c>
-      <c r="K2" t="str">
+      <c r="L2" t="str">
         <v>6282237563999</v>
       </c>
-      <c r="L2" t="str">
+      <c r="M2" t="str">
         <v>tesym21@gmail.com</v>
       </c>
-      <c r="M2" t="str">
+      <c r="N2" t="str">
         <v>Komang Adi</v>
       </c>
-      <c r="N2" t="str">
+      <c r="O2" t="str">
         <v>6282237563999</v>
       </c>
-      <c r="O2" t="str">
+      <c r="P2" t="str">
         <v>agungtoyotagianyarcustomercare@gmail.com</v>
       </c>
-      <c r="P2" t="str">
-        <v/>
+      <c r="Q2" t="str">
+        <v>SAMSAT:2026-10-22 | ASURANSI:2026-10-22 | SERVICE:2026-10-22</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(ui): ultra-clean main page, slim sticky navbar, AccuCare drawer menu, and fix 0-data table crash
</commit_message>
<xml_diff>
--- a/data/pelanggan_agung_toyota_gianyar.xlsx
+++ b/data/pelanggan_agung_toyota_gianyar.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q2"/>
+  <dimension ref="A1:Q3"/>
   <cols>
     <col min="1" max="1" width="5.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
@@ -491,16 +491,16 @@
         <v>DK 1288 KA</v>
       </c>
       <c r="G2" t="str">
-        <v>1989-10-21</v>
+        <v>1989-10-23</v>
       </c>
       <c r="H2" t="str">
-        <v>2026-10-24</v>
+        <v>2026-10-26</v>
       </c>
       <c r="I2" t="str">
-        <v>2026-10-24</v>
+        <v>2026-10-26</v>
       </c>
       <c r="J2" t="str">
-        <v>2026-10-27</v>
+        <v>2026-10-28</v>
       </c>
       <c r="K2" t="str">
         <v>I Made Putra</v>
@@ -518,15 +518,68 @@
         <v>6282237563999</v>
       </c>
       <c r="P2" t="str">
-        <v>agungtoyotagianyarcustomercare@gmail.com</v>
+        <v>tesym21@gmail.com</v>
       </c>
       <c r="Q2" t="str">
-        <v>SAMSAT:2026-10-22 | ASURANSI:2026-10-22 | SERVICE:2026-10-22</v>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="str">
+        <v>I Nengah Andika</v>
+      </c>
+      <c r="C3" t="str">
+        <v>6281805411412</v>
+      </c>
+      <c r="D3" t="str">
+        <v>andicka.nengah@gmail.com</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Toyota Zenix Hybrid Q TSS</v>
+      </c>
+      <c r="F3" t="str">
+        <v>DK 1945 KL</v>
+      </c>
+      <c r="G3" t="str">
+        <v>1989-10-23</v>
+      </c>
+      <c r="H3" t="str">
+        <v>2026-10-26</v>
+      </c>
+      <c r="I3" t="str">
+        <v>2026-10-26</v>
+      </c>
+      <c r="J3" t="str">
+        <v>2026-10-28</v>
+      </c>
+      <c r="K3" t="str">
+        <v>I Made Putra</v>
+      </c>
+      <c r="L3" t="str">
+        <v>6281805411412</v>
+      </c>
+      <c r="M3" t="str">
+        <v>made.putra@agungtoyota-gianyar.com</v>
+      </c>
+      <c r="N3" t="str">
+        <v>Komang Adi</v>
+      </c>
+      <c r="O3" t="str">
+        <v>6281999003301</v>
+      </c>
+      <c r="P3" t="str">
+        <v>andicka.nengah@gmail.com</v>
+      </c>
+      <c r="Q3" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Q2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add daily, weekly, monthly report analytics with failure reasons, charts, and Excel export
</commit_message>
<xml_diff>
--- a/data/pelanggan_agung_toyota_gianyar.xlsx
+++ b/data/pelanggan_agung_toyota_gianyar.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q3"/>
+  <dimension ref="A1:Q4"/>
   <cols>
     <col min="1" max="1" width="5.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
@@ -577,9 +577,62 @@
         <v/>
       </c>
     </row>
+    <row r="4">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="str">
+        <v>I Wayan Sudarma</v>
+      </c>
+      <c r="C4" t="str">
+        <v>6282237563999</v>
+      </c>
+      <c r="D4" t="str">
+        <v>tesym21@gmail.com</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Toyota Zenix Hybrid Q TSS</v>
+      </c>
+      <c r="F4" t="str">
+        <v>DK 1288 KA</v>
+      </c>
+      <c r="G4" t="str">
+        <v>1989-10-23</v>
+      </c>
+      <c r="H4" t="str">
+        <v>2026-10-26</v>
+      </c>
+      <c r="I4" t="str">
+        <v>2026-10-26</v>
+      </c>
+      <c r="J4" t="str">
+        <v>2026-10-28</v>
+      </c>
+      <c r="K4" t="str">
+        <v>I Made Putra</v>
+      </c>
+      <c r="L4" t="str">
+        <v>6282237563999</v>
+      </c>
+      <c r="M4" t="str">
+        <v>tesym21@gmail.com</v>
+      </c>
+      <c r="N4" t="str">
+        <v>Komang Adi</v>
+      </c>
+      <c r="O4" t="str">
+        <v>6282237563999</v>
+      </c>
+      <c r="P4" t="str">
+        <v>tesym21@gmail.com</v>
+      </c>
+      <c r="Q4" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Q3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: prevent reminder auto-retry loops, record failure reason, display issue banner and status badges
</commit_message>
<xml_diff>
--- a/data/pelanggan_agung_toyota_gianyar.xlsx
+++ b/data/pelanggan_agung_toyota_gianyar.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q4"/>
+  <dimension ref="A1:Q2"/>
   <cols>
     <col min="1" max="1" width="5.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
@@ -476,19 +476,19 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>I Wayan Sudarma</v>
+        <v>I Nengah Andika</v>
       </c>
       <c r="C2" t="str">
-        <v>6282237563999</v>
+        <v>6281805411412</v>
       </c>
       <c r="D2" t="str">
-        <v>tesym21@gmail.com</v>
+        <v>andicka.nengah@gmail.com</v>
       </c>
       <c r="E2" t="str">
         <v>Toyota Zenix Hybrid Q TSS</v>
       </c>
       <c r="F2" t="str">
-        <v>DK 1288 KA</v>
+        <v>DK 1945 KL</v>
       </c>
       <c r="G2" t="str">
         <v>1989-10-23</v>
@@ -506,133 +506,27 @@
         <v>I Made Putra</v>
       </c>
       <c r="L2" t="str">
-        <v>6282237563999</v>
+        <v>6281805411412</v>
       </c>
       <c r="M2" t="str">
-        <v>tesym21@gmail.com</v>
+        <v>made.putra@agungtoyota-gianyar.com</v>
       </c>
       <c r="N2" t="str">
         <v>Komang Adi</v>
       </c>
       <c r="O2" t="str">
-        <v>6282237563999</v>
+        <v>6281999003301</v>
       </c>
       <c r="P2" t="str">
-        <v>tesym21@gmail.com</v>
+        <v>andicka.nengah@gmail.com</v>
       </c>
       <c r="Q2" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3" t="str">
-        <v>I Nengah Andika</v>
-      </c>
-      <c r="C3" t="str">
-        <v>6281805411412</v>
-      </c>
-      <c r="D3" t="str">
-        <v>andicka.nengah@gmail.com</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Toyota Zenix Hybrid Q TSS</v>
-      </c>
-      <c r="F3" t="str">
-        <v>DK 1945 KL</v>
-      </c>
-      <c r="G3" t="str">
-        <v>1989-10-23</v>
-      </c>
-      <c r="H3" t="str">
-        <v>2026-10-26</v>
-      </c>
-      <c r="I3" t="str">
-        <v>2026-10-26</v>
-      </c>
-      <c r="J3" t="str">
-        <v>2026-10-28</v>
-      </c>
-      <c r="K3" t="str">
-        <v>I Made Putra</v>
-      </c>
-      <c r="L3" t="str">
-        <v>6281805411412</v>
-      </c>
-      <c r="M3" t="str">
-        <v>made.putra@agungtoyota-gianyar.com</v>
-      </c>
-      <c r="N3" t="str">
-        <v>Komang Adi</v>
-      </c>
-      <c r="O3" t="str">
-        <v>6281999003301</v>
-      </c>
-      <c r="P3" t="str">
-        <v>andicka.nengah@gmail.com</v>
-      </c>
-      <c r="Q3" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4" t="str">
-        <v>I Wayan Sudarma</v>
-      </c>
-      <c r="C4" t="str">
-        <v>6282237563999</v>
-      </c>
-      <c r="D4" t="str">
-        <v>tesym21@gmail.com</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Toyota Zenix Hybrid Q TSS</v>
-      </c>
-      <c r="F4" t="str">
-        <v>DK 1288 KA</v>
-      </c>
-      <c r="G4" t="str">
-        <v>1989-10-23</v>
-      </c>
-      <c r="H4" t="str">
-        <v>2026-10-26</v>
-      </c>
-      <c r="I4" t="str">
-        <v>2026-10-26</v>
-      </c>
-      <c r="J4" t="str">
-        <v>2026-10-28</v>
-      </c>
-      <c r="K4" t="str">
-        <v>I Made Putra</v>
-      </c>
-      <c r="L4" t="str">
-        <v>6282237563999</v>
-      </c>
-      <c r="M4" t="str">
-        <v>tesym21@gmail.com</v>
-      </c>
-      <c r="N4" t="str">
-        <v>Komang Adi</v>
-      </c>
-      <c r="O4" t="str">
-        <v>6282237563999</v>
-      </c>
-      <c r="P4" t="str">
-        <v>tesym21@gmail.com</v>
-      </c>
-      <c r="Q4" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Q4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add menu Pencapaian Teknisi & FO with fully editable sub-menu KPI Teknisi matching sheet KPI OKT
</commit_message>
<xml_diff>
--- a/data/pelanggan_agung_toyota_gianyar.xlsx
+++ b/data/pelanggan_agung_toyota_gianyar.xlsx
@@ -491,37 +491,37 @@
         <v>DK 1945 KL</v>
       </c>
       <c r="G2" t="str">
-        <v>1989-10-23</v>
+        <v>1989-10-29</v>
       </c>
       <c r="H2" t="str">
-        <v>2026-10-26</v>
+        <v>2026-11-01</v>
       </c>
       <c r="I2" t="str">
-        <v>2026-10-26</v>
+        <v>2026-11-01</v>
       </c>
       <c r="J2" t="str">
-        <v>2026-10-28</v>
+        <v>2026-11-03</v>
       </c>
       <c r="K2" t="str">
-        <v>I Made Putra</v>
+        <v>vivo booking</v>
       </c>
       <c r="L2" t="str">
-        <v>6281805411412</v>
+        <v>6285338175251</v>
       </c>
       <c r="M2" t="str">
         <v>made.putra@agungtoyota-gianyar.com</v>
       </c>
       <c r="N2" t="str">
-        <v>Komang Adi</v>
+        <v>mdp</v>
       </c>
       <c r="O2" t="str">
-        <v>6281999003301</v>
+        <v>6282237563999</v>
       </c>
       <c r="P2" t="str">
-        <v>andicka.nengah@gmail.com</v>
+        <v>tesym21@gmail.com</v>
       </c>
       <c r="Q2" t="str">
-        <v/>
+        <v>SERVICE:2026-10-28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Revert "feat: add menu Pencapaian Teknisi & FO with fully editable sub-menu KPI Teknisi matching sheet KPI OKT"
This reverts commit d5d0a3bf64e67896943a5fe4438465264c35a99b.
</commit_message>
<xml_diff>
--- a/data/pelanggan_agung_toyota_gianyar.xlsx
+++ b/data/pelanggan_agung_toyota_gianyar.xlsx
@@ -491,37 +491,37 @@
         <v>DK 1945 KL</v>
       </c>
       <c r="G2" t="str">
-        <v>1989-10-29</v>
+        <v>1989-10-23</v>
       </c>
       <c r="H2" t="str">
-        <v>2026-11-01</v>
+        <v>2026-10-26</v>
       </c>
       <c r="I2" t="str">
-        <v>2026-11-01</v>
+        <v>2026-10-26</v>
       </c>
       <c r="J2" t="str">
-        <v>2026-11-03</v>
+        <v>2026-10-28</v>
       </c>
       <c r="K2" t="str">
-        <v>vivo booking</v>
+        <v>I Made Putra</v>
       </c>
       <c r="L2" t="str">
-        <v>6285338175251</v>
+        <v>6281805411412</v>
       </c>
       <c r="M2" t="str">
         <v>made.putra@agungtoyota-gianyar.com</v>
       </c>
       <c r="N2" t="str">
-        <v>mdp</v>
+        <v>Komang Adi</v>
       </c>
       <c r="O2" t="str">
-        <v>6282237563999</v>
+        <v>6281999003301</v>
       </c>
       <c r="P2" t="str">
-        <v>tesym21@gmail.com</v>
+        <v>andicka.nengah@gmail.com</v>
       </c>
       <c r="Q2" t="str">
-        <v>SERVICE:2026-10-28</v>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: ensure KPI menu is completely purged and bump cache buster
</commit_message>
<xml_diff>
--- a/data/pelanggan_agung_toyota_gianyar.xlsx
+++ b/data/pelanggan_agung_toyota_gianyar.xlsx
@@ -491,37 +491,37 @@
         <v>DK 1945 KL</v>
       </c>
       <c r="G2" t="str">
-        <v>1989-10-23</v>
+        <v>1989-10-29</v>
       </c>
       <c r="H2" t="str">
-        <v>2026-10-26</v>
+        <v>2026-11-01</v>
       </c>
       <c r="I2" t="str">
-        <v>2026-10-26</v>
+        <v>2026-11-01</v>
       </c>
       <c r="J2" t="str">
-        <v>2026-10-28</v>
+        <v>2026-11-03</v>
       </c>
       <c r="K2" t="str">
-        <v>I Made Putra</v>
+        <v>vivo booking</v>
       </c>
       <c r="L2" t="str">
-        <v>6281805411412</v>
+        <v>6285338175251</v>
       </c>
       <c r="M2" t="str">
         <v>made.putra@agungtoyota-gianyar.com</v>
       </c>
       <c r="N2" t="str">
-        <v>Komang Adi</v>
+        <v>mdp</v>
       </c>
       <c r="O2" t="str">
-        <v>6281999003301</v>
+        <v>6282237563999</v>
       </c>
       <c r="P2" t="str">
-        <v>andicka.nengah@gmail.com</v>
+        <v>tesym21@gmail.com</v>
       </c>
       <c r="Q2" t="str">
-        <v/>
+        <v>SERVICE:2026-10-28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: accurate status display in customer table (differentiate GAGAL, PARSIAL, TERKIRIM, and BELUM DIKIRIM) and clear obsolete logs
</commit_message>
<xml_diff>
--- a/data/pelanggan_agung_toyota_gianyar.xlsx
+++ b/data/pelanggan_agung_toyota_gianyar.xlsx
@@ -398,25 +398,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Q2"/>
-  <cols>
-    <col min="1" max="1" width="5.83203125" customWidth="1"/>
-    <col min="2" max="2" width="24.83203125" customWidth="1"/>
-    <col min="3" max="3" width="16.83203125" customWidth="1"/>
-    <col min="4" max="4" width="25.83203125" customWidth="1"/>
-    <col min="5" max="5" width="24.83203125" customWidth="1"/>
-    <col min="6" max="6" width="14.83203125" customWidth="1"/>
-    <col min="7" max="7" width="16.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="18.83203125" customWidth="1"/>
-    <col min="10" max="10" width="18.83203125" customWidth="1"/>
-    <col min="11" max="11" width="18.83203125" customWidth="1"/>
-    <col min="12" max="12" width="16.83203125" customWidth="1"/>
-    <col min="13" max="13" width="28.83203125" customWidth="1"/>
-    <col min="14" max="14" width="18.83203125" customWidth="1"/>
-    <col min="15" max="15" width="16.83203125" customWidth="1"/>
-    <col min="16" max="16" width="28.83203125" customWidth="1"/>
-    <col min="17" max="17" width="34.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -521,7 +502,7 @@
         <v>tesym21@gmail.com</v>
       </c>
       <c r="Q2" t="str">
-        <v>SERVICE:2026-10-28</v>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: set synchronized test customer dates for tomorrow Oct 31 auto-dispatch and ensure Vercel copies fresh excel
</commit_message>
<xml_diff>
--- a/data/pelanggan_agung_toyota_gianyar.xlsx
+++ b/data/pelanggan_agung_toyota_gianyar.xlsx
@@ -472,16 +472,16 @@
         <v>DK 1945 KL</v>
       </c>
       <c r="G2" t="str">
-        <v>1989-10-29</v>
+        <v>1990-10-31</v>
       </c>
       <c r="H2" t="str">
-        <v>2026-11-01</v>
+        <v>2026-11-03</v>
       </c>
       <c r="I2" t="str">
-        <v>2026-11-01</v>
+        <v>2026-11-03</v>
       </c>
       <c r="J2" t="str">
-        <v>2026-11-03</v>
+        <v>2026-11-05</v>
       </c>
       <c r="K2" t="str">
         <v>vivo booking</v>

</xml_diff>

<commit_message>
chore: save user contact details in customer table
</commit_message>
<xml_diff>
--- a/data/pelanggan_agung_toyota_gianyar.xlsx
+++ b/data/pelanggan_agung_toyota_gianyar.xlsx
@@ -460,10 +460,10 @@
         <v>I Nengah Andika</v>
       </c>
       <c r="C2" t="str">
-        <v>6281805411412</v>
+        <v>6282237563999</v>
       </c>
       <c r="D2" t="str">
-        <v>andicka.nengah@gmail.com</v>
+        <v>tesym21@gmail.com</v>
       </c>
       <c r="E2" t="str">
         <v>Toyota Zenix Hybrid Q TSS</v>

</xml_diff>